<commit_message>
Remove SLL1069F's untimed tutorials from the complementary workbook
Removed Meetings row 178, the Thursday and Friday tutorials with no time that the last correction added. The Humanities handbook (p. 274) puts the tutorials at the 2nd and 5th periods too, which rows 153 and 155 already hold, and an untimed meeting would have made SLL1069F conditional in every plan. Shrank the CourseMeetings table to A2:G177, checked every other cell on every sheet was unchanged, and updated the manifest's fingerprint.
</commit_message>
<xml_diff>
--- a/data/sources/2026/2026_Complementary_Studies_Course_Details.xlsx
+++ b/data/sources/2026/2026_Complementary_Studies_Course_Details.xlsx
@@ -407,7 +407,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CourseMeetings" displayName="CourseMeetings" ref="A2:G178" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CourseMeetings" displayName="CourseMeetings" ref="A2:G177" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="7">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Kind"/>
@@ -9987,7 +9987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G178"/>
+  <dimension ref="A1:G177"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14569,27 +14569,7 @@
       <c r="F177" s="14" t="n"/>
       <c r="G177" s="14" t="n"/>
     </row>
-    <row r="178" ht="23" customHeight="1">
-      <c r="A178" s="14" t="inlineStr">
-        <is>
-          <t>SLL1069F</t>
-        </is>
-      </c>
-      <c r="B178" s="14" t="inlineStr">
-        <is>
-          <t>tutorial</t>
-        </is>
-      </c>
-      <c r="C178" s="14" t="inlineStr">
-        <is>
-          <t>thu,fri</t>
-        </is>
-      </c>
-      <c r="D178" s="16" t="n"/>
-      <c r="E178" s="16" t="n"/>
-      <c r="F178" s="14" t="n"/>
-      <c r="G178" s="14" t="n"/>
-    </row>
+    <row r="178" ht="23" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>